<commit_message>
feat: corte autonomo, features avanzadas de forma temporal, firma v2 y backtest de recall
</commit_message>
<xml_diff>
--- a/entregables/sospechosos.xlsx
+++ b/entregables/sospechosos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,17 +496,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUM_009931</t>
+          <t>SUM_007851</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_1538</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -516,29 +516,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>11881.28629009992</v>
+        <v>6957.855979261882</v>
       </c>
       <c r="I2" t="n">
-        <v>7924.817955496646</v>
+        <v>4640.889938167676</v>
       </c>
       <c r="J2" t="n">
-        <v>4384.12363355924</v>
+        <v>4248.770288903381</v>
       </c>
       <c r="K2" t="b">
         <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -548,22 +548,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUM_004030</t>
+          <t>SUM_001565</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SED_1137</t>
+          <t>SED_1538</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -573,17 +573,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MODERADO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>12285.17634359619</v>
+        <v>10896.59096525143</v>
       </c>
       <c r="I3" t="n">
-        <v>8194.212621178662</v>
+        <v>7268.026173822706</v>
       </c>
       <c r="J3" t="n">
-        <v>4359.855182862025</v>
+        <v>4235.169453522302</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
@@ -600,12 +600,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SUM_009955</t>
+          <t>SUM_011487</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SED_1207</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -629,13 +629,13 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>11443.49503876674</v>
+        <v>10724.08910141574</v>
       </c>
       <c r="I4" t="n">
-        <v>7632.811190857416</v>
+        <v>7152.967430644296</v>
       </c>
       <c r="J4" t="n">
-        <v>4257.079127525951</v>
+        <v>3958.090301474524</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
@@ -652,17 +652,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SUM_017526</t>
+          <t>SUM_009931</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SED_1482</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -677,17 +677,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MODERADO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>10167.65443136746</v>
+        <v>10676.20538048489</v>
       </c>
       <c r="I5" t="n">
-        <v>6781.825505722097</v>
+        <v>7121.028988783421</v>
       </c>
       <c r="J5" t="n">
-        <v>4140.59764749003</v>
+        <v>3939.455979973907</v>
       </c>
       <c r="K5" t="b">
         <v>0</v>
@@ -704,22 +704,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SUM_011487</t>
+          <t>SUM_005240</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_1019</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -729,20 +729,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>10771.39841983561</v>
+        <v>8631.953132551876</v>
       </c>
       <c r="I6" t="n">
-        <v>7184.522746030352</v>
+        <v>5757.512739412102</v>
       </c>
       <c r="J6" t="n">
-        <v>3975.551416599198</v>
+        <v>3892.111288678839</v>
       </c>
       <c r="K6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -756,17 +756,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SUM_006162</t>
+          <t>SUM_002297</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SED_1019</t>
+          <t>SED_0974</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -776,29 +776,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>10786.25885254287</v>
+        <v>6136.693658813418</v>
       </c>
       <c r="I7" t="n">
-        <v>7194.434654646094</v>
+        <v>4093.17467042855</v>
       </c>
       <c r="J7" t="n">
-        <v>3879.579278435554</v>
+        <v>3854.018022294531</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -808,12 +808,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SUM_011528</t>
+          <t>SUM_006050</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SED_1886</t>
+          <t>SED_0090</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -828,29 +828,29 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>6101.11848763978</v>
+        <v>10484.06335133136</v>
       </c>
       <c r="I8" t="n">
-        <v>4069.446031255733</v>
+        <v>6992.870255338018</v>
       </c>
       <c r="J8" t="n">
-        <v>3794.322584237284</v>
+        <v>3828.068978639672</v>
       </c>
       <c r="K8" t="b">
         <v>0</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -860,17 +860,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SUM_002297</t>
+          <t>SUM_019051</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SED_0974</t>
+          <t>SED_2738</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -880,29 +880,29 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>6026.60637740069</v>
+        <v>10168.31889135011</v>
       </c>
       <c r="I9" t="n">
-        <v>4019.74645372626</v>
+        <v>6782.268700530523</v>
       </c>
       <c r="J9" t="n">
-        <v>3784.880080891718</v>
+        <v>3748.869320241996</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -912,12 +912,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SUM_007851</t>
+          <t>SUM_018243</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_1207</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -932,29 +932,29 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>6120.902670734291</v>
+        <v>9153.2253071294</v>
       </c>
       <c r="I10" t="n">
-        <v>4082.642081379772</v>
+        <v>6105.20127985531</v>
       </c>
       <c r="J10" t="n">
-        <v>3737.690099679825</v>
+        <v>3684.62867803928</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>6160.910527307609</v>
+        <v>6037.459382261938</v>
       </c>
       <c r="I11" t="n">
-        <v>4109.327321714176</v>
+        <v>4026.985407968713</v>
       </c>
       <c r="J11" t="n">
-        <v>3728.548964315873</v>
+        <v>3653.837014359216</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
@@ -1016,17 +1016,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SUM_006050</t>
+          <t>SUM_002580</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SED_0090</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1045,13 +1045,13 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>9995.030604773117</v>
+        <v>9387.442275350422</v>
       </c>
       <c r="I12" t="n">
-        <v>6666.68541338367</v>
+        <v>6261.423997658732</v>
       </c>
       <c r="J12" t="n">
-        <v>3649.507382443209</v>
+        <v>3597.28592585602</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SUM_014910</t>
+          <t>SUM_009955</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1097,13 +1097,13 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>9513.601824337105</v>
+        <v>9319.514386211655</v>
       </c>
       <c r="I13" t="n">
-        <v>6345.57241683285</v>
+        <v>6216.116095603174</v>
       </c>
       <c r="J13" t="n">
-        <v>3636.964427561679</v>
+        <v>3466.939954779331</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
@@ -1120,12 +1120,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SUM_005714</t>
+          <t>SUM_005743</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SED_2738</t>
+          <t>SED_1207</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1149,13 +1149,13 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>9705.710625082811</v>
+        <v>9488.574270479261</v>
       </c>
       <c r="I14" t="n">
-        <v>6473.708986930235</v>
+        <v>6328.879038409667</v>
       </c>
       <c r="J14" t="n">
-        <v>3564.329809630944</v>
+        <v>3464.187889159118</v>
       </c>
       <c r="K14" t="b">
         <v>0</v>
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SUM_000944</t>
+          <t>SUM_011741</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SED_1942</t>
+          <t>SED_0035</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1201,13 +1201,13 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>5955.306486616822</v>
+        <v>5783.921313403998</v>
       </c>
       <c r="I15" t="n">
-        <v>3972.18942657342</v>
+        <v>3857.875516040467</v>
       </c>
       <c r="J15" t="n">
-        <v>3561.407027097492</v>
+        <v>3459.791944890361</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -1224,49 +1224,49 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SUM_001565</t>
+          <t>SUM_008448</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_0933</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>8905.923369568485</v>
+        <v>5459.81179702205</v>
       </c>
       <c r="I16" t="n">
-        <v>5940.25088750218</v>
+        <v>3641.694468613708</v>
       </c>
       <c r="J16" t="n">
-        <v>3461.458242351904</v>
+        <v>3443.410015568488</v>
       </c>
       <c r="K16" t="b">
         <v>0</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1276,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SUM_000475</t>
+          <t>SUM_006162</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SED_2362</t>
+          <t>SED_1019</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1296,29 +1296,29 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>5802.651988800329</v>
+        <v>9477.395821429083</v>
       </c>
       <c r="I17" t="n">
-        <v>3870.36887652982</v>
+        <v>6321.423012893199</v>
       </c>
       <c r="J17" t="n">
-        <v>3381.111461478355</v>
+        <v>3408.810130092495</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SUM_004099</t>
+          <t>SUM_004030</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SED_2195</t>
+          <t>SED_1137</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1348,29 +1348,29 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>MODERADO</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>5384.924699352855</v>
+        <v>9418.976501972855</v>
       </c>
       <c r="I18" t="n">
-        <v>3591.744774468355</v>
+        <v>6282.457326815895</v>
       </c>
       <c r="J18" t="n">
-        <v>3361.659714132808</v>
+        <v>3342.676765139625</v>
       </c>
       <c r="K18" t="b">
         <v>0</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -1380,17 +1380,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SUM_005907</t>
+          <t>SUM_009490</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SED_2475</t>
+          <t>SED_1538</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LLAVE_10</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1400,29 +1400,29 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>6336.601882372112</v>
+        <v>8806.488964485772</v>
       </c>
       <c r="I19" t="n">
-        <v>4226.513455542199</v>
+        <v>5873.92813931201</v>
       </c>
       <c r="J19" t="n">
-        <v>3358.650302867386</v>
+        <v>3329.588818246519</v>
       </c>
       <c r="K19" t="b">
         <v>0</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -1432,49 +1432,49 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SUM_013056</t>
+          <t>SUM_000944</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SED_2475</t>
+          <t>SED_1942</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LLAVE_10</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>POT_BAJA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>7980.794588739604</v>
+        <v>5549.949695728284</v>
       </c>
       <c r="I20" t="n">
-        <v>5323.189990689317</v>
+        <v>3701.816447050766</v>
       </c>
       <c r="J20" t="n">
-        <v>3278.974922882162</v>
+        <v>3318.994562382808</v>
       </c>
       <c r="K20" t="b">
         <v>0</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SUM_008448</t>
+          <t>SUM_011374</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SED_0933</t>
+          <t>SED_1041</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1504,29 +1504,29 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>5176.278345887276</v>
+        <v>8366.640626134278</v>
       </c>
       <c r="I21" t="n">
-        <v>3452.577656706814</v>
+        <v>5580.549297631564</v>
       </c>
       <c r="J21" t="n">
-        <v>3264.590312310824</v>
+        <v>3263.995037154881</v>
       </c>
       <c r="K21" t="b">
         <v>0</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1536,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SUM_008563</t>
+          <t>SUM_009540</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_0938</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1561,17 +1561,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>8476.246598250085</v>
+        <v>7503.445552682207</v>
       </c>
       <c r="I22" t="n">
-        <v>5653.656481032807</v>
+        <v>5004.798183639032</v>
       </c>
       <c r="J22" t="n">
-        <v>3246.702044669191</v>
+        <v>3258.490915676685</v>
       </c>
       <c r="K22" t="b">
         <v>0</v>
@@ -1588,12 +1588,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SUM_006458</t>
+          <t>SUM_000990</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SED_2556</t>
+          <t>SED_1041</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1603,34 +1603,34 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>8774.200692123983</v>
+        <v>5145.457306318125</v>
       </c>
       <c r="I23" t="n">
-        <v>5852.391861646697</v>
+        <v>3432.02002331419</v>
       </c>
       <c r="J23" t="n">
-        <v>3214.71653816049</v>
+        <v>3229.965618244596</v>
       </c>
       <c r="K23" t="b">
         <v>0</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -1640,17 +1640,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SUM_005743</t>
+          <t>SUM_005907</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SED_1207</t>
+          <t>SED_2475</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1660,29 +1660,29 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>8776.638069717324</v>
+        <v>6061.944958420453</v>
       </c>
       <c r="I24" t="n">
-        <v>5854.017592501456</v>
+        <v>4043.317287266442</v>
       </c>
       <c r="J24" t="n">
-        <v>3204.266778333594</v>
+        <v>3213.071240471007</v>
       </c>
       <c r="K24" t="b">
         <v>0</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -1692,12 +1692,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SUM_012471</t>
+          <t>SUM_005029</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_2154</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1721,16 +1721,16 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>8635.010088560613</v>
+        <v>9017.733418256897</v>
       </c>
       <c r="I25" t="n">
-        <v>5759.55172906993</v>
+        <v>6014.828189977351</v>
       </c>
       <c r="J25" t="n">
-        <v>3172.33075987259</v>
+        <v>3205.978852713172</v>
       </c>
       <c r="K25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>5039.592326276375</v>
+        <v>5092.241424015827</v>
       </c>
       <c r="I26" t="n">
-        <v>3361.408081626343</v>
+        <v>3396.525029818557</v>
       </c>
       <c r="J26" t="n">
-        <v>3163.177978898836</v>
+        <v>3196.223998456806</v>
       </c>
       <c r="K26" t="b">
         <v>0</v>
@@ -1796,22 +1796,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SUM_010217</t>
+          <t>SUM_014910</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_1207</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1825,13 +1825,13 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>8662.615097611506</v>
+        <v>8269.31387745091</v>
       </c>
       <c r="I27" t="n">
-        <v>5777.964270106875</v>
+        <v>5515.632356259757</v>
       </c>
       <c r="J27" t="n">
-        <v>3149.035963069152</v>
+        <v>3161.284334571853</v>
       </c>
       <c r="K27" t="b">
         <v>0</v>
@@ -1848,17 +1848,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SUM_011741</t>
+          <t>SUM_004099</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SED_0035</t>
+          <t>SED_2195</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1877,13 +1877,13 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>5220.240599246135</v>
+        <v>5053.515482074392</v>
       </c>
       <c r="I28" t="n">
-        <v>3481.900479697173</v>
+        <v>3370.694826543619</v>
       </c>
       <c r="J28" t="n">
-        <v>3122.612739181966</v>
+        <v>3154.770096019637</v>
       </c>
       <c r="K28" t="b">
         <v>0</v>
@@ -1900,17 +1900,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SUM_018799</t>
+          <t>SUM_002895</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SED_0063</t>
+          <t>SED_0212</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1929,13 +1929,13 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>8517.658937278997</v>
+        <v>8439.36346316148</v>
       </c>
       <c r="I29" t="n">
-        <v>5681.278511165091</v>
+        <v>5629.055429928708</v>
       </c>
       <c r="J29" t="n">
-        <v>3109.33620708597</v>
+        <v>3120.145175775967</v>
       </c>
       <c r="K29" t="b">
         <v>0</v>
@@ -1952,17 +1952,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SUM_000990</t>
+          <t>SUM_013499</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SED_1041</t>
+          <t>SED_0090</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1981,13 +1981,13 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>4936.473034155502</v>
+        <v>5168.314986355304</v>
       </c>
       <c r="I30" t="n">
-        <v>3292.62751378172</v>
+        <v>3447.266095898988</v>
       </c>
       <c r="J30" t="n">
-        <v>3098.779608206131</v>
+        <v>3065.196138570381</v>
       </c>
       <c r="K30" t="b">
         <v>0</v>
@@ -2004,49 +2004,49 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SUM_005240</t>
+          <t>SUM_017150</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SED_1019</t>
+          <t>SED_1270</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>6816.919074307418</v>
+        <v>4884.043017872074</v>
       </c>
       <c r="I31" t="n">
-        <v>4546.885022563048</v>
+        <v>3257.656692920673</v>
       </c>
       <c r="J31" t="n">
-        <v>3073.720081155984</v>
+        <v>3059.284505578766</v>
       </c>
       <c r="K31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2056,12 +2056,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SUM_001082</t>
+          <t>SUM_018118</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SED_2105</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2071,34 +2071,34 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>POT_BAJA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>5714.160281879617</v>
+        <v>4958.686766890946</v>
       </c>
       <c r="I32" t="n">
-        <v>3811.344908013705</v>
+        <v>3307.444073516261</v>
       </c>
       <c r="J32" t="n">
-        <v>3050.998951006357</v>
+        <v>2999.520629226256</v>
       </c>
       <c r="K32" t="b">
         <v>0</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2108,12 +2108,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SUM_016429</t>
+          <t>SUM_014340</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SED_1159</t>
+          <t>SED_2362</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2128,29 +2128,29 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>8061.171996427995</v>
+        <v>5959.136664166298</v>
       </c>
       <c r="I33" t="n">
-        <v>5376.801721617473</v>
+        <v>3974.744154998921</v>
       </c>
       <c r="J33" t="n">
-        <v>3043.797162590237</v>
+        <v>2986.633767103137</v>
       </c>
       <c r="K33" t="b">
         <v>0</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2160,17 +2160,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SUM_016085</t>
+          <t>SUM_017321</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SED_2002</t>
+          <t>SED_0035</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2180,29 +2180,29 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>5158.142373163886</v>
+        <v>8118.019667590993</v>
       </c>
       <c r="I34" t="n">
-        <v>3440.480962900312</v>
+        <v>5414.719118283193</v>
       </c>
       <c r="J34" t="n">
-        <v>3012.397671872287</v>
+        <v>2984.040817943008</v>
       </c>
       <c r="K34" t="b">
         <v>0</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SUM_001518</t>
+          <t>SUM_013724</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SED_0044</t>
+          <t>SED_2315</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2232,29 +2232,29 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>5963.763278422727</v>
+        <v>7032.103963043591</v>
       </c>
       <c r="I35" t="n">
-        <v>3977.830106707959</v>
+        <v>4690.413343350076</v>
       </c>
       <c r="J35" t="n">
-        <v>2974.320425158363</v>
+        <v>2937.373771453356</v>
       </c>
       <c r="K35" t="b">
         <v>0</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -2264,22 +2264,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SUM_017009</t>
+          <t>SUM_011954</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SED_0837</t>
+          <t>SED_0933</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>POT_BAJA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2289,17 +2289,17 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>5666.04235124327</v>
+        <v>7721.300032363034</v>
       </c>
       <c r="I36" t="n">
-        <v>3779.250248279261</v>
+        <v>5150.107121586144</v>
       </c>
       <c r="J36" t="n">
-        <v>2950.413302894709</v>
+        <v>2923.755054675239</v>
       </c>
       <c r="K36" t="b">
         <v>0</v>
@@ -2316,17 +2316,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SUM_016262</t>
+          <t>SUM_000731</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SED_1523</t>
+          <t>SED_2181</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2345,20 +2345,20 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>6825.452989085968</v>
+        <v>7348.027538323156</v>
       </c>
       <c r="I37" t="n">
-        <v>4552.57714372034</v>
+        <v>4901.134368061546</v>
       </c>
       <c r="J37" t="n">
-        <v>2944.009078799763</v>
+        <v>2907.24106150566</v>
       </c>
       <c r="K37" t="b">
         <v>0</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -2368,12 +2368,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SUM_015909</t>
+          <t>SUM_000475</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SED_2738</t>
+          <t>SED_2362</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2388,29 +2388,29 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>8045.028848843588</v>
+        <v>4981.201008812113</v>
       </c>
       <c r="I38" t="n">
-        <v>5366.034242178674</v>
+        <v>3322.46107287768</v>
       </c>
       <c r="J38" t="n">
-        <v>2917.764720916882</v>
+        <v>2902.465261630171</v>
       </c>
       <c r="K38" t="b">
         <v>0</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2420,22 +2420,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SUM_005952</t>
+          <t>SUM_004081</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SED_2475</t>
+          <t>SED_1565</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>LLAVE_10</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>POT_BAJA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2449,13 +2449,13 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>7759.081411277064</v>
+        <v>7684.452228508026</v>
       </c>
       <c r="I39" t="n">
-        <v>5175.307301321802</v>
+        <v>5125.529636414853</v>
       </c>
       <c r="J39" t="n">
-        <v>2895.093518786156</v>
+        <v>2884.544878535373</v>
       </c>
       <c r="K39" t="b">
         <v>0</v>
@@ -2472,17 +2472,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SUM_016528</t>
+          <t>SUM_002389</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_2738</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2501,20 +2501,20 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>7237.710594248574</v>
+        <v>7616.071680441203</v>
       </c>
       <c r="I40" t="n">
-        <v>4827.552966363799</v>
+        <v>5079.919810854283</v>
       </c>
       <c r="J40" t="n">
-        <v>2874.309741458171</v>
+        <v>2861.322262192136</v>
       </c>
       <c r="K40" t="b">
         <v>0</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2524,12 +2524,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SUM_003643</t>
+          <t>SUM_015875</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_0539</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>7664.792802646253</v>
+        <v>7036.357146518349</v>
       </c>
       <c r="I41" t="n">
-        <v>5112.416799365051</v>
+        <v>4693.250216727739</v>
       </c>
       <c r="J41" t="n">
-        <v>2851.085773372743</v>
+        <v>2854.458991209573</v>
       </c>
       <c r="K41" t="b">
         <v>0</v>
@@ -2576,17 +2576,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SUM_003931</t>
+          <t>SUM_014334</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SED_2181</t>
+          <t>SED_1538</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2605,13 +2605,13 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>6744.592344793261</v>
+        <v>7707.681122318587</v>
       </c>
       <c r="I42" t="n">
-        <v>4498.643093977105</v>
+        <v>5141.023308586497</v>
       </c>
       <c r="J42" t="n">
-        <v>2845.714410107075</v>
+        <v>2854.155611507502</v>
       </c>
       <c r="K42" t="b">
         <v>0</v>
@@ -2628,17 +2628,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SUM_007710</t>
+          <t>SUM_011528</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SED_1041</t>
+          <t>SED_1886</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2657,13 +2657,13 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>4562.517554180758</v>
+        <v>4589.135962958863</v>
       </c>
       <c r="I43" t="n">
-        <v>3043.199208638566</v>
+        <v>3060.953687293562</v>
       </c>
       <c r="J43" t="n">
-        <v>2840.333140332651</v>
+        <v>2854.011483577402</v>
       </c>
       <c r="K43" t="b">
         <v>0</v>
@@ -2680,12 +2680,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SUM_010889</t>
+          <t>SUM_004297</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_0063</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2709,13 +2709,13 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>6998.922150898258</v>
+        <v>7833.907888724081</v>
       </c>
       <c r="I44" t="n">
-        <v>4668.281074649139</v>
+        <v>5225.216561778962</v>
       </c>
       <c r="J44" t="n">
-        <v>2823.523110851856</v>
+        <v>2853.960604512855</v>
       </c>
       <c r="K44" t="b">
         <v>0</v>
@@ -2732,17 +2732,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SUM_010946</t>
+          <t>SUM_016262</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SED_2642</t>
+          <t>SED_1523</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2752,7 +2752,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2761,20 +2761,20 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>7651.776207976513</v>
+        <v>6613.226242400466</v>
       </c>
       <c r="I45" t="n">
-        <v>5103.734730720334</v>
+        <v>4411.021903681111</v>
       </c>
       <c r="J45" t="n">
-        <v>2811.06718274885</v>
+        <v>2852.469737747189</v>
       </c>
       <c r="K45" t="b">
         <v>0</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2784,22 +2784,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SUM_000996</t>
+          <t>SUM_014878</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SED_1159</t>
+          <t>SED_2475</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_10</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2813,13 +2813,13 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>7243.88084535551</v>
+        <v>7556.602722918652</v>
       </c>
       <c r="I46" t="n">
-        <v>4831.668523852126</v>
+        <v>5040.254016186741</v>
       </c>
       <c r="J46" t="n">
-        <v>2792.321125042849</v>
+        <v>2827.33762670947</v>
       </c>
       <c r="K46" t="b">
         <v>0</v>
@@ -2836,17 +2836,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SUM_013336</t>
+          <t>SUM_005714</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_2738</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>LLAVE_10</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2865,20 +2865,20 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>7399.879226802223</v>
+        <v>7643.331341830802</v>
       </c>
       <c r="I47" t="n">
-        <v>4935.719444277083</v>
+        <v>5098.102005001145</v>
       </c>
       <c r="J47" t="n">
-        <v>2777.813712318279</v>
+        <v>2806.940655758687</v>
       </c>
       <c r="K47" t="b">
         <v>0</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -2888,17 +2888,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SUM_004297</t>
+          <t>SUM_003643</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SED_0063</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2917,13 +2917,13 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>7597.111644945005</v>
+        <v>7499.180900639142</v>
       </c>
       <c r="I48" t="n">
-        <v>5067.273467178318</v>
+        <v>5001.953660726308</v>
       </c>
       <c r="J48" t="n">
-        <v>2767.69367865139</v>
+        <v>2789.482837732962</v>
       </c>
       <c r="K48" t="b">
         <v>0</v>
@@ -2940,12 +2940,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SUM_017150</t>
+          <t>SUM_016085</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SED_1270</t>
+          <t>SED_2002</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2969,13 +2969,13 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>4413.92805813709</v>
+        <v>4751.581412081981</v>
       </c>
       <c r="I49" t="n">
-        <v>2944.09001477744</v>
+        <v>3169.304801858682</v>
       </c>
       <c r="J49" t="n">
-        <v>2764.812199152474</v>
+        <v>2774.962718737003</v>
       </c>
       <c r="K49" t="b">
         <v>0</v>
@@ -2992,17 +2992,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SUM_002580</t>
+          <t>SUM_001518</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_0044</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3012,29 +3012,29 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>7211.405872147523</v>
+        <v>5548.976341268216</v>
       </c>
       <c r="I50" t="n">
-        <v>4810.007716722398</v>
+        <v>3701.1672196259</v>
       </c>
       <c r="J50" t="n">
-        <v>2763.424593046925</v>
+        <v>2767.452848148528</v>
       </c>
       <c r="K50" t="b">
         <v>0</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3044,17 +3044,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SUM_018341</t>
+          <t>SUM_013344</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_0044</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3064,29 +3064,29 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>7029.416327578637</v>
+        <v>5296.048186348301</v>
       </c>
       <c r="I51" t="n">
-        <v>4688.620690494951</v>
+        <v>3532.464140294317</v>
       </c>
       <c r="J51" t="n">
-        <v>2738.118297140565</v>
+        <v>2759.613030382295</v>
       </c>
       <c r="K51" t="b">
         <v>0</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3096,12 +3096,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SUM_002895</t>
+          <t>SUM_012633</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SED_0212</t>
+          <t>SED_1207</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3125,13 +3125,13 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>7360.823205266113</v>
+        <v>7439.54640436752</v>
       </c>
       <c r="I52" t="n">
-        <v>4909.669077912497</v>
+        <v>4962.177451713136</v>
       </c>
       <c r="J52" t="n">
-        <v>2721.3944646303</v>
+        <v>2750.087432923928</v>
       </c>
       <c r="K52" t="b">
         <v>0</v>
@@ -3148,49 +3148,49 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SUM_010398</t>
+          <t>SUM_004118</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SED_2743</t>
+          <t>SED_0670</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>7399.228998311606</v>
+        <v>4981.80475944569</v>
       </c>
       <c r="I53" t="n">
-        <v>4935.285741873841</v>
+        <v>3322.863774550276</v>
       </c>
       <c r="J53" t="n">
-        <v>2712.813420672936</v>
+        <v>2749.863556669656</v>
       </c>
       <c r="K53" t="b">
         <v>0</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3200,49 +3200,49 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SUM_009486</t>
+          <t>SUM_010398</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SED_2295</t>
+          <t>SED_2743</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>4771.825440520587</v>
+        <v>7477.575834499323</v>
       </c>
       <c r="I54" t="n">
-        <v>3182.807568827232</v>
+        <v>4987.543081611048</v>
       </c>
       <c r="J54" t="n">
-        <v>2690.826542738741</v>
+        <v>2741.538082218861</v>
       </c>
       <c r="K54" t="b">
         <v>0</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -3252,17 +3252,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>SUM_009540</t>
+          <t>SUM_012384</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SED_0938</t>
+          <t>SED_2329</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_13</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3281,13 +3281,13 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>6194.554286861757</v>
+        <v>6611.629917885751</v>
       </c>
       <c r="I55" t="n">
-        <v>4131.767709336792</v>
+        <v>4409.957155229796</v>
       </c>
       <c r="J55" t="n">
-        <v>2690.084005899095</v>
+        <v>2725.361741267513</v>
       </c>
       <c r="K55" t="b">
         <v>0</v>
@@ -3304,49 +3304,49 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SUM_003889</t>
+          <t>SUM_006785</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_2195</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MUY_ALTA</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MODERADO</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>6714.706927041841</v>
+        <v>5438.501110311087</v>
       </c>
       <c r="I56" t="n">
-        <v>4478.709520336908</v>
+        <v>3627.480240577495</v>
       </c>
       <c r="J56" t="n">
-        <v>2689.358471479121</v>
+        <v>2720.300814643505</v>
       </c>
       <c r="K56" t="b">
         <v>0</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3356,12 +3356,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>SUM_010160</t>
+          <t>SUM_002074</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SED_0044</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3376,29 +3376,29 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>5397.106213500778</v>
+        <v>6898.955794601119</v>
       </c>
       <c r="I57" t="n">
-        <v>3599.869844405019</v>
+        <v>4601.603514998947</v>
       </c>
       <c r="J57" t="n">
-        <v>2682.86113550527</v>
+        <v>2707.357708297088</v>
       </c>
       <c r="K57" t="b">
         <v>0</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -3408,12 +3408,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SUM_010229</t>
+          <t>SUM_015688</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SED_2074</t>
+          <t>SED_2362</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3428,29 +3428,29 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>7310.730449122739</v>
+        <v>5298.192524752312</v>
       </c>
       <c r="I58" t="n">
-        <v>4876.257209564867</v>
+        <v>3533.894414009792</v>
       </c>
       <c r="J58" t="n">
-        <v>2677.282688197079</v>
+        <v>2692.366859666118</v>
       </c>
       <c r="K58" t="b">
         <v>0</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3460,22 +3460,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SUM_018516</t>
+          <t>SUM_006458</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SED_1159</t>
+          <t>SED_2556</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3489,13 +3489,13 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>7035.633393829806</v>
+        <v>7346.859046325235</v>
       </c>
       <c r="I59" t="n">
-        <v>4692.767473684481</v>
+        <v>4900.354983898932</v>
       </c>
       <c r="J59" t="n">
-        <v>2674.420232205276</v>
+        <v>2691.763057227094</v>
       </c>
       <c r="K59" t="b">
         <v>0</v>
@@ -3512,17 +3512,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SUM_013344</t>
+          <t>SUM_013189</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SED_0044</t>
+          <t>SED_1137</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3532,29 +3532,29 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>5111.923289982826</v>
+        <v>6798.963908158466</v>
       </c>
       <c r="I60" t="n">
-        <v>3409.652834418545</v>
+        <v>4534.908926741697</v>
       </c>
       <c r="J60" t="n">
-        <v>2663.67102884656</v>
+        <v>2689.062488381113</v>
       </c>
       <c r="K60" t="b">
         <v>0</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -3564,49 +3564,49 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>SUM_001336</t>
+          <t>SUM_010160</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SED_0151</t>
+          <t>SED_0044</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="H61" t="n">
-        <v>6098.924546328009</v>
+        <v>5406.93600071179</v>
       </c>
       <c r="I61" t="n">
-        <v>4067.982672400783</v>
+        <v>3606.426312474764</v>
       </c>
       <c r="J61" t="n">
-        <v>2646.734901853139</v>
+        <v>2687.747449214039</v>
       </c>
       <c r="K61" t="b">
         <v>0</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3616,12 +3616,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>SUM_012079</t>
+          <t>SUM_012246</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SED_1019</t>
+          <t>SED_1206</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3636,29 +3636,29 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H62" t="n">
-        <v>7332.668126761369</v>
+        <v>4315.619770327784</v>
       </c>
       <c r="I62" t="n">
-        <v>4890.889640549833</v>
+        <v>2878.518386808632</v>
       </c>
       <c r="J62" t="n">
-        <v>2640.20361807553</v>
+        <v>2683.956270674251</v>
       </c>
       <c r="K62" t="b">
         <v>0</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3668,12 +3668,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SUM_011954</t>
+          <t>SUM_010609</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SED_0933</t>
+          <t>SED_1538</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3697,13 +3697,13 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>6969.430480371552</v>
+        <v>6537.321351297423</v>
       </c>
       <c r="I63" t="n">
-        <v>4648.610130407826</v>
+        <v>4360.393341315381</v>
       </c>
       <c r="J63" t="n">
-        <v>2639.051391577363</v>
+        <v>2672.967648828436</v>
       </c>
       <c r="K63" t="b">
         <v>0</v>
@@ -3720,17 +3720,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SUM_006848</t>
+          <t>SUM_000032</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SED_0061</t>
+          <t>SED_1565</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3745,17 +3745,17 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H64" t="n">
-        <v>4961.476603179367</v>
+        <v>7292.846405521293</v>
       </c>
       <c r="I64" t="n">
-        <v>3309.304894320638</v>
+        <v>4864.328552482703</v>
       </c>
       <c r="J64" t="n">
-        <v>2624.267338561046</v>
+        <v>2672.25914645374</v>
       </c>
       <c r="K64" t="b">
         <v>0</v>
@@ -3772,17 +3772,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SUM_018439</t>
+          <t>SUM_010946</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SED_2738</t>
+          <t>SED_2642</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3801,20 +3801,20 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>7172.073624769764</v>
+        <v>7270.043679509253</v>
       </c>
       <c r="I65" t="n">
-        <v>4783.773107721433</v>
+        <v>4849.119134232672</v>
       </c>
       <c r="J65" t="n">
-        <v>2599.462420150571</v>
+        <v>2670.828399727015</v>
       </c>
       <c r="K65" t="b">
         <v>0</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3824,17 +3824,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SUM_002389</t>
+          <t>SUM_008803</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SED_2738</t>
+          <t>SED_2470</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_10</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3853,20 +3853,20 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>6895.508774651985</v>
+        <v>5722.582320820836</v>
       </c>
       <c r="I66" t="n">
-        <v>4599.304352692874</v>
+        <v>3816.962407987497</v>
       </c>
       <c r="J66" t="n">
-        <v>2590.610172002735</v>
+        <v>2663.420610923041</v>
       </c>
       <c r="K66" t="b">
         <v>0</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3876,12 +3876,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SUM_009490</t>
+          <t>SUM_018297</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_1777</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3891,34 +3891,34 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_BAJA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>6850.588319768504</v>
+        <v>4405.798667273562</v>
       </c>
       <c r="I67" t="n">
-        <v>4569.342409285593</v>
+        <v>2938.667711071466</v>
       </c>
       <c r="J67" t="n">
-        <v>2590.094912955282</v>
+        <v>2639.810640744347</v>
       </c>
       <c r="K67" t="b">
         <v>0</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -3928,22 +3928,22 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SUM_014340</t>
+          <t>SUM_001082</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SED_2362</t>
+          <t>SED_2105</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_BAJA</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3957,13 +3957,13 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>5162.875218502972</v>
+        <v>4934.912978856316</v>
       </c>
       <c r="I68" t="n">
-        <v>3443.637770741482</v>
+        <v>3291.586956897163</v>
       </c>
       <c r="J68" t="n">
-        <v>2587.558958941616</v>
+        <v>2634.930344803981</v>
       </c>
       <c r="K68" t="b">
         <v>0</v>
@@ -3980,49 +3980,49 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SUM_012731</t>
+          <t>SUM_005469</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SED_2181</t>
+          <t>SED_1523</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>MODERADO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H69" t="n">
-        <v>6010.662254607415</v>
+        <v>5684.406217090219</v>
       </c>
       <c r="I69" t="n">
-        <v>4009.111723823146</v>
+        <v>3791.498946799176</v>
       </c>
       <c r="J69" t="n">
-        <v>2576.667188425988</v>
+        <v>2624.754348847905</v>
       </c>
       <c r="K69" t="b">
         <v>0</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4032,22 +4032,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SUM_013987</t>
+          <t>SUM_018422</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SED_2738</t>
+          <t>SED_1594</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -4061,13 +4061,13 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>7036.051282674339</v>
+        <v>6274.601487325013</v>
       </c>
       <c r="I70" t="n">
-        <v>4693.046205543785</v>
+        <v>4185.159192045784</v>
       </c>
       <c r="J70" t="n">
-        <v>2566.51297261763</v>
+        <v>2618.189815396204</v>
       </c>
       <c r="K70" t="b">
         <v>0</v>
@@ -4084,27 +4084,27 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SUM_011118</t>
+          <t>SUM_011532</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SED_0498</t>
+          <t>SED_0515</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -4113,20 +4113,20 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>5633.219653703149</v>
+        <v>7082.123347378488</v>
       </c>
       <c r="I71" t="n">
-        <v>3757.35750902</v>
+        <v>4723.776272701451</v>
       </c>
       <c r="J71" t="n">
-        <v>2562.398869124856</v>
+        <v>2615.973345382809</v>
       </c>
       <c r="K71" t="b">
         <v>0</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -4136,12 +4136,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SUM_018243</t>
+          <t>SUM_010227</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SED_1207</t>
+          <t>SED_2002</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4156,29 +4156,29 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MODERADO</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>6358.312397804559</v>
+        <v>5239.824370252482</v>
       </c>
       <c r="I72" t="n">
-        <v>4240.994369335641</v>
+        <v>3494.962854958406</v>
       </c>
       <c r="J72" t="n">
-        <v>2559.537148794471</v>
+        <v>2610.681627865932</v>
       </c>
       <c r="K72" t="b">
         <v>0</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4188,12 +4188,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SUM_013475</t>
+          <t>SUM_018232</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SED_0061</t>
+          <t>SED_2413</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4208,29 +4208,29 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>6828.587820859715</v>
+        <v>5583.400032475945</v>
       </c>
       <c r="I73" t="n">
-        <v>4554.668076513431</v>
+        <v>3724.127821661456</v>
       </c>
       <c r="J73" t="n">
-        <v>2559.314973646928</v>
+        <v>2608.19311246592</v>
       </c>
       <c r="K73" t="b">
         <v>0</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4240,27 +4240,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SUM_003734</t>
+          <t>SUM_010229</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SED_0670</t>
+          <t>SED_2074</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>LLAVE_10</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>POT_BAJA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4269,20 +4269,20 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>6757.460044008161</v>
+        <v>7115.901350248994</v>
       </c>
       <c r="I74" t="n">
-        <v>4507.225849353444</v>
+        <v>4746.30620061608</v>
       </c>
       <c r="J74" t="n">
-        <v>2559.058810978206</v>
+        <v>2605.933788493862</v>
       </c>
       <c r="K74" t="b">
         <v>0</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4292,27 +4292,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SUM_011532</t>
+          <t>SUM_000739</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_2407</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4321,20 +4321,20 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>6868.970817204059</v>
+        <v>6924.20878834252</v>
       </c>
       <c r="I75" t="n">
-        <v>4581.603535075108</v>
+        <v>4618.447261824461</v>
       </c>
       <c r="J75" t="n">
-        <v>2537.239707166298</v>
+        <v>2593.044760786061</v>
       </c>
       <c r="K75" t="b">
         <v>0</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4344,22 +4344,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SUM_004744</t>
+          <t>SUM_003940</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SED_2295</t>
+          <t>SED_2362</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4369,20 +4369,20 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H76" t="n">
-        <v>6823.908294963444</v>
+        <v>5995.630065599324</v>
       </c>
       <c r="I76" t="n">
-        <v>4551.546832740617</v>
+        <v>3999.085253754749</v>
       </c>
       <c r="J76" t="n">
-        <v>2517.245077457424</v>
+        <v>2590.52316986656</v>
       </c>
       <c r="K76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -4396,17 +4396,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SUM_014334</t>
+          <t>SUM_001065</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_2362</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -4425,20 +4425,20 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>6793.577703874238</v>
+        <v>5627.569000752997</v>
       </c>
       <c r="I77" t="n">
-        <v>4531.316328484117</v>
+        <v>3753.588523502249</v>
       </c>
       <c r="J77" t="n">
-        <v>2515.662962441306</v>
+        <v>2585.968196377046</v>
       </c>
       <c r="K77" t="b">
         <v>0</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4448,12 +4448,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SUM_004082</t>
+          <t>SUM_001195</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>SED_1538</t>
+          <t>SED_2642</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4463,12 +4463,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4477,20 +4477,20 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>6170.817100620721</v>
+        <v>6904.689885387177</v>
       </c>
       <c r="I78" t="n">
-        <v>4115.935006114021</v>
+        <v>4605.428153553247</v>
       </c>
       <c r="J78" t="n">
-        <v>2514.463298964145</v>
+        <v>2583.157581194693</v>
       </c>
       <c r="K78" t="b">
         <v>0</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4500,12 +4500,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SUM_013768</t>
+          <t>SUM_018799</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SED_2363</t>
+          <t>SED_0063</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4529,13 +4529,13 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>6738.798122744614</v>
+        <v>7039.227267560163</v>
       </c>
       <c r="I79" t="n">
-        <v>4494.778347870658</v>
+        <v>4695.164587462628</v>
       </c>
       <c r="J79" t="n">
-        <v>2503.405410883442</v>
+        <v>2569.640833719935</v>
       </c>
       <c r="K79" t="b">
         <v>0</v>
@@ -4552,12 +4552,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SUM_010536</t>
+          <t>SUM_010274</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SED_1207</t>
+          <t>SED_2789</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4581,20 +4581,20 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>6188.780162210782</v>
+        <v>6886.608025157372</v>
       </c>
       <c r="I80" t="n">
-        <v>4127.916368194592</v>
+        <v>4593.367552779968</v>
       </c>
       <c r="J80" t="n">
-        <v>2489.209928500032</v>
+        <v>2569.550790358962</v>
       </c>
       <c r="K80" t="b">
         <v>0</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4604,17 +4604,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SUM_006641</t>
+          <t>SUM_015876</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>SED_1019</t>
+          <t>SED_0853</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_10</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4624,29 +4624,29 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MODERADO</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>6792.619056205438</v>
+        <v>5089.047622557711</v>
       </c>
       <c r="I81" t="n">
-        <v>4530.676910489027</v>
+        <v>3394.394764245993</v>
       </c>
       <c r="J81" t="n">
-        <v>2487.928496246876</v>
+        <v>2568.788808633626</v>
       </c>
       <c r="K81" t="b">
         <v>0</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4656,17 +4656,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SUM_000731</t>
+          <t>SUM_006364</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SED_2181</t>
+          <t>SED_1159</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -4685,13 +4685,13 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>6279.815897204818</v>
+        <v>6293.525880420064</v>
       </c>
       <c r="I82" t="n">
-        <v>4188.637203435614</v>
+        <v>4197.781762240183</v>
       </c>
       <c r="J82" t="n">
-        <v>2484.60400288812</v>
+        <v>2565.830403387873</v>
       </c>
       <c r="K82" t="b">
         <v>0</v>
@@ -4708,49 +4708,49 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SUM_016916</t>
+          <t>SUM_019587</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SED_2475</t>
+          <t>SED_0090</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>LLAVE_05</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>POT_BAJA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H83" t="n">
-        <v>6703.778566432625</v>
+        <v>4591.16252804968</v>
       </c>
       <c r="I83" t="n">
-        <v>4471.420303810561</v>
+        <v>3062.305406209137</v>
       </c>
       <c r="J83" t="n">
-        <v>2480.866273911275</v>
+        <v>2560.942001379785</v>
       </c>
       <c r="K83" t="b">
         <v>0</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4760,12 +4760,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SUM_012633</t>
+          <t>SUM_001764</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>SED_1207</t>
+          <t>SED_0063</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -4789,13 +4789,13 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>6706.454021953255</v>
+        <v>6005.093528315483</v>
       </c>
       <c r="I84" t="n">
-        <v>4473.204832642821</v>
+        <v>4005.397383386427</v>
       </c>
       <c r="J84" t="n">
-        <v>2479.094009606323</v>
+        <v>2550.15092537023</v>
       </c>
       <c r="K84" t="b">
         <v>0</v>
@@ -4812,12 +4812,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SUM_011374</t>
+          <t>SUM_012663</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SED_1041</t>
+          <t>SED_2738</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4841,20 +4841,20 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>6350.927185404393</v>
+        <v>6858.83139924383</v>
       </c>
       <c r="I85" t="n">
-        <v>4236.068432664731</v>
+        <v>4574.840543295635</v>
       </c>
       <c r="J85" t="n">
-        <v>2477.624621492768</v>
+        <v>2547.881408773974</v>
       </c>
       <c r="K85" t="b">
         <v>0</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -4864,22 +4864,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SUM_012607</t>
+          <t>SUM_013290</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SED_1207</t>
+          <t>SED_2738</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -4889,17 +4889,17 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H86" t="n">
-        <v>4326.991767123411</v>
+        <v>6785.887209647562</v>
       </c>
       <c r="I86" t="n">
-        <v>2886.103508671315</v>
+        <v>4526.186768834924</v>
       </c>
       <c r="J86" t="n">
-        <v>2477.598561252347</v>
+        <v>2546.376430539181</v>
       </c>
       <c r="K86" t="b">
         <v>0</v>
@@ -4916,17 +4916,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SUM_018545</t>
+          <t>SUM_006382</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SED_0450</t>
+          <t>SED_0938</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_05</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4941,17 +4941,17 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MUY ALTO</t>
         </is>
       </c>
       <c r="H87" t="n">
-        <v>6717.800369167673</v>
+        <v>4480.05373592691</v>
       </c>
       <c r="I87" t="n">
-        <v>4480.772846234839</v>
+        <v>2988.195841863249</v>
       </c>
       <c r="J87" t="n">
-        <v>2461.344499242131</v>
+        <v>2544.927916214495</v>
       </c>
       <c r="K87" t="b">
         <v>0</v>
@@ -4968,17 +4968,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SUM_000317</t>
+          <t>SUM_012607</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SED_2789</t>
+          <t>SED_1207</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_16</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4988,29 +4988,29 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>MUY ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H88" t="n">
-        <v>5664.656438213219</v>
+        <v>4414.807195195694</v>
       </c>
       <c r="I88" t="n">
-        <v>3778.325844288217</v>
+        <v>2944.676399195529</v>
       </c>
       <c r="J88" t="n">
-        <v>2461.067710659662</v>
+        <v>2527.880925989151</v>
       </c>
       <c r="K88" t="b">
         <v>0</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -5020,12 +5020,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SUM_004253</t>
+          <t>SUM_011118</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SED_0501</t>
+          <t>SED_0498</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -5049,20 +5049,20 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>6681.86100857302</v>
+        <v>5553.71434389873</v>
       </c>
       <c r="I89" t="n">
-        <v>4456.801292718204</v>
+        <v>3704.327467380453</v>
       </c>
       <c r="J89" t="n">
-        <v>2459.556993599062</v>
+        <v>2526.234059574364</v>
       </c>
       <c r="K89" t="b">
         <v>0</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -5072,12 +5072,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SUM_003499</t>
+          <t>SUM_004253</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SED_0515</t>
+          <t>SED_0501</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5087,12 +5087,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_MEDIA</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -5101,20 +5101,20 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>6101.229705985391</v>
+        <v>6841.719473686626</v>
       </c>
       <c r="I90" t="n">
-        <v>4069.520213892256</v>
+        <v>4563.426888948979</v>
       </c>
       <c r="J90" t="n">
-        <v>2453.407489254886</v>
+        <v>2518.400032290186</v>
       </c>
       <c r="K90" t="b">
         <v>0</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -5124,12 +5124,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SUM_015411</t>
+          <t>SUM_002164</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SED_2181</t>
+          <t>SED_0742</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5139,34 +5139,34 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_BAJA</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H91" t="n">
-        <v>5798.131112396847</v>
+        <v>4167.280215051721</v>
       </c>
       <c r="I91" t="n">
-        <v>3867.353451968697</v>
+        <v>2779.575903439498</v>
       </c>
       <c r="J91" t="n">
-        <v>2453.286238942052</v>
+        <v>2513.95328368642</v>
       </c>
       <c r="K91" t="b">
         <v>0</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -5176,12 +5176,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SUM_005469</t>
+          <t>SUM_004400</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SED_1523</t>
+          <t>SED_2295</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5191,12 +5191,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>POT_MEDIA</t>
+          <t>POT_ALTA</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -5205,20 +5205,20 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>5302.978465003874</v>
+        <v>6262.30012798449</v>
       </c>
       <c r="I92" t="n">
-        <v>3537.086636157584</v>
+        <v>4176.954185365656</v>
       </c>
       <c r="J92" t="n">
-        <v>2448.631441225656</v>
+        <v>2511.719510754935</v>
       </c>
       <c r="K92" t="b">
         <v>0</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -5228,17 +5228,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SUM_003296</t>
+          <t>SUM_001643</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SED_0035</t>
+          <t>SED_2074</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -5248,29 +5248,29 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>4360.65912222596</v>
+        <v>6100.979848899451</v>
       </c>
       <c r="I93" t="n">
-        <v>2908.559634524716</v>
+        <v>4069.353559215934</v>
       </c>
       <c r="J93" t="n">
-        <v>2448.419605063566</v>
+        <v>2510.776571417148</v>
       </c>
       <c r="K93" t="b">
         <v>0</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -5280,22 +5280,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SUM_012246</t>
+          <t>SUM_012733</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>SED_1206</t>
+          <t>SED_2475</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>LLAVE_08</t>
+          <t>LLAVE_10</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_BAJA</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -5305,17 +5305,17 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="H94" t="n">
-        <v>3936.29725884148</v>
+        <v>6560.566843860965</v>
       </c>
       <c r="I94" t="n">
-        <v>2625.510271647267</v>
+        <v>4375.898084855265</v>
       </c>
       <c r="J94" t="n">
-        <v>2448.049242832861</v>
+        <v>2508.908620890374</v>
       </c>
       <c r="K94" t="b">
         <v>0</v>
@@ -5332,17 +5332,17 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>SUM_008803</t>
+          <t>SUM_000996</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SED_2470</t>
+          <t>SED_1159</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>LLAVE_10</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>MANIPULACIÓN</t>
+          <t>CLANDESTINA</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -5361,20 +5361,20 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>5255.117552983887</v>
+        <v>6503.533223477966</v>
       </c>
       <c r="I95" t="n">
-        <v>3505.163407840253</v>
+        <v>4337.856660059803</v>
       </c>
       <c r="J95" t="n">
-        <v>2445.851823313413</v>
+        <v>2506.937040382018</v>
       </c>
       <c r="K95" t="b">
         <v>0</v>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>REVISAR MEDIDOR</t>
+          <t>REVISAR RED / ACOMETIDA</t>
         </is>
       </c>
     </row>
@@ -5384,12 +5384,12 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SUM_006630</t>
+          <t>SUM_003806</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SED_0038</t>
+          <t>SED_2475</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5399,34 +5399,34 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>POT_ALTA</t>
+          <t>POT_BAJA</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>CLANDESTINA</t>
+          <t>MANIPULACIÓN</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>CRÍTICO</t>
         </is>
       </c>
       <c r="H96" t="n">
-        <v>6467.308071341185</v>
+        <v>4111.464014422341</v>
       </c>
       <c r="I96" t="n">
-        <v>4313.694483584571</v>
+        <v>2742.346497619702</v>
       </c>
       <c r="J96" t="n">
-        <v>2439.636731885035</v>
+        <v>2500.049716888795</v>
       </c>
       <c r="K96" t="b">
         <v>0</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>REVISAR RED / ACOMETIDA</t>
+          <t>REVISAR MEDIDOR</t>
         </is>
       </c>
     </row>
@@ -5436,17 +5436,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SUM_013623</t>
+          <t>SUM_013768</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SED_1137</t>
+          <t>SED_2363</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>LLAVE_16</t>
+          <t>LLAVE_08</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -5465,226 +5465,18 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>6634.735115881549</v>
+        <v>6681.477446929048</v>
       </c>
       <c r="I97" t="n">
-        <v>4425.368322292993</v>
+        <v>4456.545457101675</v>
       </c>
       <c r="J97" t="n">
-        <v>2433.16797596184</v>
+        <v>2482.111273950053</v>
       </c>
       <c r="K97" t="b">
         <v>0</v>
       </c>
       <c r="L97" t="inlineStr">
-        <is>
-          <t>REVISAR RED / ACOMETIDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>SUM_009770</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>SED_1594</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>LLAVE_16</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>POT_MEDIA</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>CLANDESTINA</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="H98" t="n">
-        <v>6551.632117785081</v>
-      </c>
-      <c r="I98" t="n">
-        <v>4369.938622562649</v>
-      </c>
-      <c r="J98" t="n">
-        <v>2430.299097965146</v>
-      </c>
-      <c r="K98" t="b">
-        <v>0</v>
-      </c>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t>REVISAR RED / ACOMETIDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>SUM_013698</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>SED_2329</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>LLAVE_08</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>POT_BAJA</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>MANIPULACIÓN</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>CRÍTICO</t>
-        </is>
-      </c>
-      <c r="H99" t="n">
-        <v>4547.227667766027</v>
-      </c>
-      <c r="I99" t="n">
-        <v>3033.00085439994</v>
-      </c>
-      <c r="J99" t="n">
-        <v>2428.892162714312</v>
-      </c>
-      <c r="K99" t="b">
-        <v>0</v>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>REVISAR MEDIDOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="n">
-        <v>99</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>SUM_013499</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>SED_0090</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>LLAVE_08</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>POT_ALTA</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>MANIPULACIÓN</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>CRÍTICO</t>
-        </is>
-      </c>
-      <c r="H100" t="n">
-        <v>4085.63544529171</v>
-      </c>
-      <c r="I100" t="n">
-        <v>2725.118842009571</v>
-      </c>
-      <c r="J100" t="n">
-        <v>2423.086445693946</v>
-      </c>
-      <c r="K100" t="b">
-        <v>0</v>
-      </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>REVISAR MEDIDOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="n">
-        <v>100</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>SUM_002211</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>SED_2661</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>LLAVE_08</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>POT_MEDIA</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>CLANDESTINA</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="H101" t="n">
-        <v>6388.207572868187</v>
-      </c>
-      <c r="I101" t="n">
-        <v>4260.93445110308</v>
-      </c>
-      <c r="J101" t="n">
-        <v>2417.526240783734</v>
-      </c>
-      <c r="K101" t="b">
-        <v>0</v>
-      </c>
-      <c r="L101" t="inlineStr">
         <is>
           <t>REVISAR RED / ACOMETIDA</t>
         </is>

</xml_diff>